<commit_message>
Financials slide, Aeon stores, competitive areas blue, expandable chart
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/empire-sushi/public/Menu Items/Empire Sushi Menu.xlsx
+++ b/empire-sushi/public/Menu Items/Empire Sushi Menu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\NAZRIN\nazrins\Empire Sushi\empire-sushi\public\Menu Items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7B66853-02BD-4B60-9349-2959BE6D2FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DD74B19-CA8F-4E27-B662-6ED26D51DCEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-852" windowWidth="23256" windowHeight="12456" xr2:uid="{C5C4E6CC-BC29-4AF0-BF6E-A7F6FD24A9CC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C5C4E6CC-BC29-4AF0-BF6E-A7F6FD24A9CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>Item</t>
   </si>
@@ -184,18 +184,6 @@
   </si>
   <si>
     <t>Cheesy Ebi</t>
-  </si>
-  <si>
-    <t>Empire Combo 1</t>
-  </si>
-  <si>
-    <t>Empire Combo 2</t>
-  </si>
-  <si>
-    <t>Empire Combo 3</t>
-  </si>
-  <si>
-    <t>Empire Combo 4</t>
   </si>
   <si>
     <t>Inari + Potato Mayo</t>
@@ -642,7 +630,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6971305B-7B1C-4C00-A465-769AFE856C55}">
-  <dimension ref="A1:B80"/>
+  <dimension ref="A1:B76"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.7265625" customWidth="1"/>
@@ -654,7 +642,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="29" x14ac:dyDescent="0.35">
@@ -729,7 +717,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -737,7 +725,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -745,7 +733,7 @@
         <v>2.8</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -753,7 +741,7 @@
         <v>2.8</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -761,7 +749,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -769,7 +757,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -777,7 +765,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -793,7 +781,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -801,7 +789,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -809,7 +797,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -817,7 +805,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -825,7 +813,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -833,7 +821,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -841,7 +829,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -849,7 +837,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
@@ -857,7 +845,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
@@ -865,7 +853,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>27</v>
       </c>
@@ -873,7 +861,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
@@ -881,7 +869,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>29</v>
       </c>
@@ -889,7 +877,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>30</v>
       </c>
@@ -897,7 +885,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
@@ -905,7 +893,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>32</v>
       </c>
@@ -913,7 +901,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>33</v>
       </c>
@@ -921,7 +909,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>34</v>
       </c>
@@ -937,7 +925,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>36</v>
       </c>
@@ -945,7 +933,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
@@ -953,7 +941,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
@@ -969,7 +957,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
@@ -1001,7 +989,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>44</v>
       </c>
@@ -1009,7 +997,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
@@ -1017,7 +1005,7 @@
         <v>2.8</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>46</v>
       </c>
@@ -1041,7 +1029,7 @@
         <v>3.4</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>49</v>
       </c>
@@ -1049,47 +1037,47 @@
         <v>3.4</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B51" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B52" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B53" s="2">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B54" s="2">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>54</v>
       </c>
       <c r="B55" s="2">
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>55</v>
       </c>
@@ -1097,103 +1085,103 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>56</v>
       </c>
       <c r="B57" s="2">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>57</v>
       </c>
       <c r="B58" s="2">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B59" s="2">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B60" s="2">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>60</v>
       </c>
       <c r="B61" s="2">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>61</v>
       </c>
       <c r="B62" s="2">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B63" s="2">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B64" s="2">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>64</v>
       </c>
       <c r="B65" s="2">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B66" s="2">
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>66</v>
       </c>
       <c r="B67" s="2">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>67</v>
       </c>
       <c r="B68" s="2">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>68</v>
       </c>
@@ -1201,7 +1189,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>69</v>
       </c>
@@ -1209,7 +1197,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>70</v>
       </c>
@@ -1217,15 +1205,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B72" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>72</v>
       </c>
@@ -1233,7 +1221,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>73</v>
       </c>
@@ -1241,51 +1229,19 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>74</v>
       </c>
       <c r="B75" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B76" s="2">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A77" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B77" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A78" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B78" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A79" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B79" s="2">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A80" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B80" s="2">
         <v>5.5</v>
       </c>
     </row>

</xml_diff>